<commit_message>
Add Report Builder executive summary deliverable
New ~2-3 page plain-language exec brief (report_builder_exec_summary.py) built on the shared walkthrough engine and single-source figures. Leads with the estimate reconciliation (~15 day core build, ~9 optional testing, ~24 total). Wired into regenerate_all.py; README updated (new row + corrected total). Includes updated estimates spreadsheet.
</commit_message>
<xml_diff>
--- a/analysis/BRYT/report-builder/deliverables/BRYT Report Builder Estimates.xlsx
+++ b/analysis/BRYT/report-builder/deliverables/BRYT Report Builder Estimates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\d55-analysis\analysis\BRYT\report-builder\deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E85246A3-9E4E-4DB9-80E2-E0D42FC7E3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573A9411-8BC1-47CA-B505-65DC1E3D18C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -780,7 +780,7 @@
       </c>
       <c r="C4" s="2">
         <f>SUMIFS('Task Detail'!$E:$E,'Task Detail'!$A:$A,$A4,'Task Detail'!$F:$F,"")</f>
-        <v>1.25</v>
+        <v>0.875</v>
       </c>
       <c r="D4" s="2">
         <f>SUMIFS('Task Detail'!$E:$E,'Task Detail'!$A:$A,$A4,'Task Detail'!$F:$F,"Yes")</f>
@@ -788,7 +788,7 @@
       </c>
       <c r="E4" s="2">
         <f t="shared" ref="E4:E11" si="0">C4+D4</f>
-        <v>1.25</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
@@ -864,7 +864,7 @@
       </c>
       <c r="C8" s="2">
         <f>SUMIFS('Task Detail'!$E:$E,'Task Detail'!$A:$A,$A8,'Task Detail'!$F:$F,"")</f>
-        <v>4.75</v>
+        <v>3.75</v>
       </c>
       <c r="D8" s="2">
         <f>SUMIFS('Task Detail'!$E:$E,'Task Detail'!$A:$A,$A8,'Task Detail'!$F:$F,"Yes")</f>
@@ -872,7 +872,7 @@
       </c>
       <c r="E8" s="2">
         <f t="shared" si="0"/>
-        <v>6.75</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
@@ -948,7 +948,7 @@
       </c>
       <c r="C12" s="3">
         <f>SUM(C4:C11)</f>
-        <v>16.5</v>
+        <v>15.125</v>
       </c>
       <c r="D12" s="3">
         <f>SUM(D4:D11)</f>
@@ -956,7 +956,7 @@
       </c>
       <c r="E12" s="3">
         <f>SUM(E4:E11)</f>
-        <v>25.5</v>
+        <v>24.125</v>
       </c>
     </row>
   </sheetData>
@@ -969,6 +969,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
@@ -1000,7 +1001,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1018,7 +1019,7 @@
       </c>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -1032,11 +1033,11 @@
         <v>26</v>
       </c>
       <c r="E3" s="2">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1050,11 +1051,11 @@
         <v>26</v>
       </c>
       <c r="E4" s="2">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -1068,11 +1069,11 @@
         <v>26</v>
       </c>
       <c r="E5" s="2">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1090,7 +1091,7 @@
       </c>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -1108,7 +1109,7 @@
       </c>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -1126,7 +1127,7 @@
       </c>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1144,7 +1145,7 @@
       </c>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -1162,7 +1163,7 @@
       </c>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -1182,7 +1183,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -1200,7 +1201,7 @@
       </c>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
@@ -1218,7 +1219,7 @@
       </c>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
@@ -1236,7 +1237,7 @@
       </c>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>8</v>
       </c>
@@ -1254,7 +1255,7 @@
       </c>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
@@ -1272,7 +1273,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>8</v>
       </c>
@@ -1290,7 +1291,7 @@
       </c>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1308,7 +1309,7 @@
       </c>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -1326,7 +1327,7 @@
       </c>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1376,7 +1377,7 @@
         <v>68</v>
       </c>
       <c r="E22" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F22" s="2"/>
     </row>
@@ -1394,7 +1395,7 @@
         <v>68</v>
       </c>
       <c r="E23" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F23" s="2"/>
     </row>
@@ -1454,7 +1455,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>11</v>
       </c>
@@ -1472,7 +1473,7 @@
       </c>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>11</v>
       </c>
@@ -1490,7 +1491,7 @@
       </c>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>11</v>
       </c>
@@ -1508,7 +1509,7 @@
       </c>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>11</v>
       </c>
@@ -1526,7 +1527,7 @@
       </c>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>11</v>
       </c>
@@ -1544,7 +1545,7 @@
       </c>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>11</v>
       </c>
@@ -1564,7 +1565,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>12</v>
       </c>
@@ -1584,7 +1585,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>12</v>
       </c>
@@ -1602,7 +1603,7 @@
       </c>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
@@ -1620,7 +1621,7 @@
       </c>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>13</v>
       </c>
@@ -1638,7 +1639,7 @@
       </c>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>13</v>
       </c>
@@ -1658,7 +1659,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
@@ -1678,7 +1679,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>13</v>
       </c>
@@ -1697,7 +1698,13 @@
       <c r="F39" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F39" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:F39" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Phase 5: Assistant (Converse loop) + query generation"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>